<commit_message>
"Final tested and approved ver of Quran_Analysis_App"
</commit_message>
<xml_diff>
--- a/موضوعات كل سورة بالقرآن.xlsx
+++ b/موضوعات كل سورة بالقرآن.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Quran_Analysis_App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183FFD3A-005F-4B68-AD2E-2053450B8382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D6E6446-8657-4725-9828-21623553258C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{44609DA0-D60F-486C-89A4-5DE82B1B4551}"/>
   </bookViews>
@@ -1598,7 +1598,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="2"/>
@@ -1639,20 +1639,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="2"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="2"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="2"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="2"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1971,7 +1974,7 @@
   <dimension ref="A1:K365"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="9" max="9" width="100.77734375" style="18" customWidth="1"/>
+    <col min="9" max="9" width="100.77734375" style="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -1999,7 +2002,7 @@
       <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="14" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2028,7 +2031,7 @@
       <c r="H2" s="5">
         <v>1</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="15" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2057,7 +2060,7 @@
       <c r="H3" s="5">
         <v>1</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="I3" s="15" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2086,7 +2089,7 @@
       <c r="H4" s="5">
         <v>1</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="15" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2115,7 +2118,7 @@
       <c r="H5" s="5">
         <v>2</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="I5" s="15" t="s">
         <v>14</v>
       </c>
     </row>
@@ -2144,7 +2147,7 @@
       <c r="H6" s="5">
         <v>2</v>
       </c>
-      <c r="I6" s="14" t="s">
+      <c r="I6" s="15" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2173,7 +2176,7 @@
       <c r="H7" s="5">
         <v>2</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="I7" s="15" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2202,7 +2205,7 @@
       <c r="H8" s="5">
         <v>2</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="I8" s="16" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2231,7 +2234,7 @@
       <c r="H9" s="5">
         <v>3</v>
       </c>
-      <c r="I9" s="15" t="s">
+      <c r="I9" s="16" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2260,7 +2263,7 @@
       <c r="H10" s="5">
         <v>3</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="I10" s="16" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2289,7 +2292,7 @@
       <c r="H11" s="5">
         <v>3</v>
       </c>
-      <c r="I11" s="15" t="s">
+      <c r="I11" s="16" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2318,7 +2321,7 @@
       <c r="H12" s="5">
         <v>4</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="16" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2347,7 +2350,7 @@
       <c r="H13" s="5">
         <v>4</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="I13" s="16" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2376,7 +2379,7 @@
       <c r="H14" s="5">
         <v>4</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="I14" s="16" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2405,7 +2408,7 @@
       <c r="H15" s="5">
         <v>5</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I15" s="16" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2434,7 +2437,7 @@
       <c r="H16" s="5">
         <v>5</v>
       </c>
-      <c r="I16" s="15" t="s">
+      <c r="I16" s="16" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2463,7 +2466,7 @@
       <c r="H17" s="7">
         <v>6</v>
       </c>
-      <c r="I17" s="16" t="s">
+      <c r="I17" s="17" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2492,7 +2495,7 @@
       <c r="H18" s="7">
         <v>6</v>
       </c>
-      <c r="I18" s="16" t="s">
+      <c r="I18" s="17" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2521,7 +2524,7 @@
       <c r="H19" s="7">
         <v>6</v>
       </c>
-      <c r="I19" s="16" t="s">
+      <c r="I19" s="17" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2550,7 +2553,7 @@
       <c r="H20" s="7">
         <v>6</v>
       </c>
-      <c r="I20" s="16" t="s">
+      <c r="I20" s="17" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2579,7 +2582,7 @@
       <c r="H21" s="5">
         <v>7</v>
       </c>
-      <c r="I21" s="15" t="s">
+      <c r="I21" s="16" t="s">
         <v>35</v>
       </c>
     </row>
@@ -2608,7 +2611,7 @@
       <c r="H22" s="5">
         <v>7</v>
       </c>
-      <c r="I22" s="15" t="s">
+      <c r="I22" s="16" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2637,7 +2640,7 @@
       <c r="H23" s="5">
         <v>7</v>
       </c>
-      <c r="I23" s="15" t="s">
+      <c r="I23" s="16" t="s">
         <v>37</v>
       </c>
     </row>
@@ -2666,7 +2669,7 @@
       <c r="H24" s="5">
         <v>7</v>
       </c>
-      <c r="I24" s="15" t="s">
+      <c r="I24" s="16" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2695,7 +2698,7 @@
       <c r="H25" s="5">
         <v>8</v>
       </c>
-      <c r="I25" s="15" t="s">
+      <c r="I25" s="16" t="s">
         <v>40</v>
       </c>
     </row>
@@ -2724,7 +2727,7 @@
       <c r="H26" s="5">
         <v>8</v>
       </c>
-      <c r="I26" s="15" t="s">
+      <c r="I26" s="16" t="s">
         <v>41</v>
       </c>
     </row>
@@ -2753,7 +2756,7 @@
       <c r="H27" s="5">
         <v>8</v>
       </c>
-      <c r="I27" s="15" t="s">
+      <c r="I27" s="16" t="s">
         <v>42</v>
       </c>
     </row>
@@ -2782,7 +2785,7 @@
       <c r="H28" s="5">
         <v>9</v>
       </c>
-      <c r="I28" s="15" t="s">
+      <c r="I28" s="16" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2811,7 +2814,7 @@
       <c r="H29" s="5">
         <v>9</v>
       </c>
-      <c r="I29" s="15" t="s">
+      <c r="I29" s="16" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2840,7 +2843,7 @@
       <c r="H30" s="5">
         <v>9</v>
       </c>
-      <c r="I30" s="15" t="s">
+      <c r="I30" s="16" t="s">
         <v>46</v>
       </c>
     </row>
@@ -2869,7 +2872,7 @@
       <c r="H31" s="5">
         <v>10</v>
       </c>
-      <c r="I31" s="15" t="s">
+      <c r="I31" s="16" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2898,7 +2901,7 @@
       <c r="H32" s="5">
         <v>10</v>
       </c>
-      <c r="I32" s="15" t="s">
+      <c r="I32" s="16" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2927,7 +2930,7 @@
       <c r="H33" s="5">
         <v>10</v>
       </c>
-      <c r="I33" s="15" t="s">
+      <c r="I33" s="16" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2956,7 +2959,7 @@
       <c r="H34" s="5">
         <v>10</v>
       </c>
-      <c r="I34" s="15" t="s">
+      <c r="I34" s="16" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2985,7 +2988,7 @@
       <c r="H35" s="5">
         <v>11</v>
       </c>
-      <c r="I35" s="15" t="s">
+      <c r="I35" s="16" t="s">
         <v>53</v>
       </c>
     </row>
@@ -3014,7 +3017,7 @@
       <c r="H36" s="5">
         <v>11</v>
       </c>
-      <c r="I36" s="15" t="s">
+      <c r="I36" s="16" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3043,7 +3046,7 @@
       <c r="H37" s="5">
         <v>11</v>
       </c>
-      <c r="I37" s="15" t="s">
+      <c r="I37" s="16" t="s">
         <v>55</v>
       </c>
     </row>
@@ -3072,7 +3075,7 @@
       <c r="H38" s="5">
         <v>11</v>
       </c>
-      <c r="I38" s="15" t="s">
+      <c r="I38" s="16" t="s">
         <v>56</v>
       </c>
     </row>
@@ -3101,7 +3104,7 @@
       <c r="H39" s="5">
         <v>11</v>
       </c>
-      <c r="I39" s="15" t="s">
+      <c r="I39" s="16" t="s">
         <v>57</v>
       </c>
     </row>
@@ -3130,7 +3133,7 @@
       <c r="H40" s="5">
         <v>11</v>
       </c>
-      <c r="I40" s="15" t="s">
+      <c r="I40" s="16" t="s">
         <v>58</v>
       </c>
     </row>
@@ -3159,7 +3162,7 @@
       <c r="H41" s="9">
         <v>12</v>
       </c>
-      <c r="I41" s="15" t="s">
+      <c r="I41" s="16" t="s">
         <v>60</v>
       </c>
     </row>
@@ -3188,7 +3191,7 @@
       <c r="H42" s="9">
         <v>12</v>
       </c>
-      <c r="I42" s="15" t="s">
+      <c r="I42" s="16" t="s">
         <v>61</v>
       </c>
     </row>
@@ -3217,7 +3220,7 @@
       <c r="H43" s="5">
         <v>13</v>
       </c>
-      <c r="I43" s="15" t="s">
+      <c r="I43" s="16" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3246,7 +3249,7 @@
       <c r="H44" s="5">
         <v>13</v>
       </c>
-      <c r="I44" s="15" t="s">
+      <c r="I44" s="16" t="s">
         <v>64</v>
       </c>
     </row>
@@ -3275,7 +3278,7 @@
       <c r="H45" s="5">
         <v>13</v>
       </c>
-      <c r="I45" s="15" t="s">
+      <c r="I45" s="16" t="s">
         <v>65</v>
       </c>
     </row>
@@ -3304,7 +3307,7 @@
       <c r="H46" s="5">
         <v>14</v>
       </c>
-      <c r="I46" s="15" t="s">
+      <c r="I46" s="16" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3333,7 +3336,7 @@
       <c r="H47" s="5">
         <v>14</v>
       </c>
-      <c r="I47" s="15" t="s">
+      <c r="I47" s="16" t="s">
         <v>68</v>
       </c>
     </row>
@@ -3362,7 +3365,7 @@
       <c r="H48" s="5">
         <v>15</v>
       </c>
-      <c r="I48" s="15" t="s">
+      <c r="I48" s="16" t="s">
         <v>70</v>
       </c>
     </row>
@@ -3391,7 +3394,7 @@
       <c r="H49" s="5">
         <v>15</v>
       </c>
-      <c r="I49" s="15" t="s">
+      <c r="I49" s="16" t="s">
         <v>71</v>
       </c>
     </row>
@@ -3420,7 +3423,7 @@
       <c r="H50" s="5">
         <v>15</v>
       </c>
-      <c r="I50" s="15" t="s">
+      <c r="I50" s="16" t="s">
         <v>72</v>
       </c>
     </row>
@@ -3449,7 +3452,7 @@
       <c r="H51" s="5">
         <v>16</v>
       </c>
-      <c r="I51" s="15" t="s">
+      <c r="I51" s="16" t="s">
         <v>74</v>
       </c>
     </row>
@@ -3478,7 +3481,7 @@
       <c r="H52" s="5">
         <v>16</v>
       </c>
-      <c r="I52" s="15" t="s">
+      <c r="I52" s="16" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3507,7 +3510,7 @@
       <c r="H53" s="5">
         <v>16</v>
       </c>
-      <c r="I53" s="15" t="s">
+      <c r="I53" s="16" t="s">
         <v>76</v>
       </c>
     </row>
@@ -3536,7 +3539,7 @@
       <c r="H54" s="5">
         <v>16</v>
       </c>
-      <c r="I54" s="15" t="s">
+      <c r="I54" s="16" t="s">
         <v>77</v>
       </c>
     </row>
@@ -3565,7 +3568,7 @@
       <c r="H55" s="5">
         <v>17</v>
       </c>
-      <c r="I55" s="15" t="s">
+      <c r="I55" s="16" t="s">
         <v>79</v>
       </c>
     </row>
@@ -3594,7 +3597,7 @@
       <c r="H56" s="5">
         <v>17</v>
       </c>
-      <c r="I56" s="15" t="s">
+      <c r="I56" s="16" t="s">
         <v>80</v>
       </c>
     </row>
@@ -3623,7 +3626,7 @@
       <c r="H57" s="5">
         <v>17</v>
       </c>
-      <c r="I57" s="15" t="s">
+      <c r="I57" s="16" t="s">
         <v>81</v>
       </c>
     </row>
@@ -3652,7 +3655,7 @@
       <c r="H58" s="11">
         <v>18</v>
       </c>
-      <c r="I58" s="17" t="s">
+      <c r="I58" s="18" t="s">
         <v>83</v>
       </c>
     </row>
@@ -3665,7 +3668,7 @@
       <c r="F59" s="11"/>
       <c r="G59" s="11"/>
       <c r="H59" s="11"/>
-      <c r="I59" s="17" t="s">
+      <c r="I59" s="18" t="s">
         <v>84</v>
       </c>
     </row>
@@ -3694,7 +3697,7 @@
       <c r="H60" s="5">
         <v>19</v>
       </c>
-      <c r="I60" s="15" t="s">
+      <c r="I60" s="16" t="s">
         <v>86</v>
       </c>
     </row>
@@ -3723,7 +3726,7 @@
       <c r="H61" s="5">
         <v>19</v>
       </c>
-      <c r="I61" s="15" t="s">
+      <c r="I61" s="16" t="s">
         <v>87</v>
       </c>
     </row>
@@ -3752,7 +3755,7 @@
       <c r="H62" s="5">
         <v>19</v>
       </c>
-      <c r="I62" s="15" t="s">
+      <c r="I62" s="16" t="s">
         <v>88</v>
       </c>
     </row>
@@ -3781,7 +3784,7 @@
       <c r="H63" s="5">
         <v>19</v>
       </c>
-      <c r="I63" s="15" t="s">
+      <c r="I63" s="16" t="s">
         <v>89</v>
       </c>
     </row>
@@ -3810,7 +3813,7 @@
       <c r="H64" s="5">
         <v>20</v>
       </c>
-      <c r="I64" s="15" t="s">
+      <c r="I64" s="16" t="s">
         <v>91</v>
       </c>
     </row>
@@ -3839,7 +3842,7 @@
       <c r="H65" s="5">
         <v>20</v>
       </c>
-      <c r="I65" s="15" t="s">
+      <c r="I65" s="16" t="s">
         <v>92</v>
       </c>
     </row>
@@ -3868,7 +3871,7 @@
       <c r="H66" s="5">
         <v>20</v>
       </c>
-      <c r="I66" s="15" t="s">
+      <c r="I66" s="16" t="s">
         <v>93</v>
       </c>
     </row>
@@ -3897,7 +3900,7 @@
       <c r="H67" s="5">
         <v>20</v>
       </c>
-      <c r="I67" s="15" t="s">
+      <c r="I67" s="16" t="s">
         <v>94</v>
       </c>
     </row>
@@ -3926,7 +3929,7 @@
       <c r="H68" s="5">
         <v>20</v>
       </c>
-      <c r="I68" s="15" t="s">
+      <c r="I68" s="16" t="s">
         <v>95</v>
       </c>
     </row>
@@ -3955,7 +3958,7 @@
       <c r="H69" s="5">
         <v>21</v>
       </c>
-      <c r="I69" s="15" t="s">
+      <c r="I69" s="16" t="s">
         <v>97</v>
       </c>
     </row>
@@ -3984,7 +3987,7 @@
       <c r="H70" s="5">
         <v>21</v>
       </c>
-      <c r="I70" s="15" t="s">
+      <c r="I70" s="16" t="s">
         <v>98</v>
       </c>
     </row>
@@ -4013,7 +4016,7 @@
       <c r="H71" s="5">
         <v>21</v>
       </c>
-      <c r="I71" s="15" t="s">
+      <c r="I71" s="16" t="s">
         <v>99</v>
       </c>
     </row>
@@ -4042,7 +4045,7 @@
       <c r="H72" s="5">
         <v>21</v>
       </c>
-      <c r="I72" s="15" t="s">
+      <c r="I72" s="16" t="s">
         <v>100</v>
       </c>
     </row>
@@ -4071,7 +4074,7 @@
       <c r="H73" s="5">
         <v>21</v>
       </c>
-      <c r="I73" s="15" t="s">
+      <c r="I73" s="16" t="s">
         <v>101</v>
       </c>
     </row>
@@ -4100,7 +4103,7 @@
       <c r="H74" s="5">
         <v>22</v>
       </c>
-      <c r="I74" s="15" t="s">
+      <c r="I74" s="16" t="s">
         <v>103</v>
       </c>
     </row>
@@ -4129,7 +4132,7 @@
       <c r="H75" s="5">
         <v>22</v>
       </c>
-      <c r="I75" s="15" t="s">
+      <c r="I75" s="16" t="s">
         <v>104</v>
       </c>
     </row>
@@ -4158,7 +4161,7 @@
       <c r="H76" s="5">
         <v>22</v>
       </c>
-      <c r="I76" s="15" t="s">
+      <c r="I76" s="16" t="s">
         <v>105</v>
       </c>
     </row>
@@ -4187,7 +4190,7 @@
       <c r="H77" s="5">
         <v>22</v>
       </c>
-      <c r="I77" s="15" t="s">
+      <c r="I77" s="16" t="s">
         <v>106</v>
       </c>
     </row>
@@ -4216,7 +4219,7 @@
       <c r="H78" s="5">
         <v>23</v>
       </c>
-      <c r="I78" s="15" t="s">
+      <c r="I78" s="16" t="s">
         <v>108</v>
       </c>
     </row>
@@ -4245,7 +4248,7 @@
       <c r="H79" s="5">
         <v>23</v>
       </c>
-      <c r="I79" s="15" t="s">
+      <c r="I79" s="16" t="s">
         <v>109</v>
       </c>
     </row>
@@ -4274,7 +4277,7 @@
       <c r="H80" s="5">
         <v>23</v>
       </c>
-      <c r="I80" s="15" t="s">
+      <c r="I80" s="16" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4303,7 +4306,7 @@
       <c r="H81" s="5">
         <v>23</v>
       </c>
-      <c r="I81" s="15" t="s">
+      <c r="I81" s="16" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4332,7 +4335,7 @@
       <c r="H82" s="5">
         <v>23</v>
       </c>
-      <c r="I82" s="15" t="s">
+      <c r="I82" s="16" t="s">
         <v>112</v>
       </c>
     </row>
@@ -4361,7 +4364,7 @@
       <c r="H83" s="5">
         <v>24</v>
       </c>
-      <c r="I83" s="15" t="s">
+      <c r="I83" s="16" t="s">
         <v>114</v>
       </c>
     </row>
@@ -4390,7 +4393,7 @@
       <c r="H84" s="5">
         <v>24</v>
       </c>
-      <c r="I84" s="15" t="s">
+      <c r="I84" s="16" t="s">
         <v>115</v>
       </c>
     </row>
@@ -4419,7 +4422,7 @@
       <c r="H85" s="5">
         <v>24</v>
       </c>
-      <c r="I85" s="15" t="s">
+      <c r="I85" s="16" t="s">
         <v>116</v>
       </c>
     </row>
@@ -4448,7 +4451,7 @@
       <c r="H86" s="5">
         <v>24</v>
       </c>
-      <c r="I86" s="15" t="s">
+      <c r="I86" s="16" t="s">
         <v>117</v>
       </c>
     </row>
@@ -4477,7 +4480,7 @@
       <c r="H87" s="5">
         <v>24</v>
       </c>
-      <c r="I87" s="15" t="s">
+      <c r="I87" s="16" t="s">
         <v>118</v>
       </c>
     </row>
@@ -4506,7 +4509,7 @@
       <c r="H88" s="5">
         <v>25</v>
       </c>
-      <c r="I88" s="15" t="s">
+      <c r="I88" s="16" t="s">
         <v>120</v>
       </c>
     </row>
@@ -4535,7 +4538,7 @@
       <c r="H89" s="5">
         <v>25</v>
       </c>
-      <c r="I89" s="15" t="s">
+      <c r="I89" s="16" t="s">
         <v>121</v>
       </c>
     </row>
@@ -4564,7 +4567,7 @@
       <c r="H90" s="5">
         <v>25</v>
       </c>
-      <c r="I90" s="15" t="s">
+      <c r="I90" s="16" t="s">
         <v>122</v>
       </c>
     </row>
@@ -4593,7 +4596,7 @@
       <c r="H91" s="5">
         <v>25</v>
       </c>
-      <c r="I91" s="15" t="s">
+      <c r="I91" s="16" t="s">
         <v>123</v>
       </c>
     </row>
@@ -4622,7 +4625,7 @@
       <c r="H92" s="5">
         <v>26</v>
       </c>
-      <c r="I92" s="15" t="s">
+      <c r="I92" s="16" t="s">
         <v>125</v>
       </c>
     </row>
@@ -4651,7 +4654,7 @@
       <c r="H93" s="5">
         <v>26</v>
       </c>
-      <c r="I93" s="15" t="s">
+      <c r="I93" s="16" t="s">
         <v>126</v>
       </c>
     </row>
@@ -4680,7 +4683,7 @@
       <c r="H94" s="5">
         <v>26</v>
       </c>
-      <c r="I94" s="15" t="s">
+      <c r="I94" s="16" t="s">
         <v>127</v>
       </c>
     </row>
@@ -4709,7 +4712,7 @@
       <c r="H95" s="5">
         <v>27</v>
       </c>
-      <c r="I95" s="15" t="s">
+      <c r="I95" s="16" t="s">
         <v>129</v>
       </c>
     </row>
@@ -4738,7 +4741,7 @@
       <c r="H96" s="5">
         <v>27</v>
       </c>
-      <c r="I96" s="15" t="s">
+      <c r="I96" s="16" t="s">
         <v>130</v>
       </c>
     </row>
@@ -4767,7 +4770,7 @@
       <c r="H97" s="5">
         <v>27</v>
       </c>
-      <c r="I97" s="15" t="s">
+      <c r="I97" s="16" t="s">
         <v>131</v>
       </c>
     </row>
@@ -4796,7 +4799,7 @@
       <c r="H98" s="5">
         <v>27</v>
       </c>
-      <c r="I98" s="15" t="s">
+      <c r="I98" s="16" t="s">
         <v>132</v>
       </c>
     </row>
@@ -4825,7 +4828,7 @@
       <c r="H99" s="9">
         <v>28</v>
       </c>
-      <c r="I99" s="15" t="s">
+      <c r="I99" s="16" t="s">
         <v>134</v>
       </c>
     </row>
@@ -4854,7 +4857,7 @@
       <c r="H100" s="9">
         <v>28</v>
       </c>
-      <c r="I100" s="15" t="s">
+      <c r="I100" s="16" t="s">
         <v>135</v>
       </c>
     </row>
@@ -4883,7 +4886,7 @@
       <c r="H101" s="9">
         <v>28</v>
       </c>
-      <c r="I101" s="15" t="s">
+      <c r="I101" s="16" t="s">
         <v>136</v>
       </c>
     </row>
@@ -4912,7 +4915,7 @@
       <c r="H102" s="9">
         <v>28</v>
       </c>
-      <c r="I102" s="15" t="s">
+      <c r="I102" s="16" t="s">
         <v>137</v>
       </c>
     </row>
@@ -4941,7 +4944,7 @@
       <c r="H103" s="9">
         <v>28</v>
       </c>
-      <c r="I103" s="15" t="s">
+      <c r="I103" s="16" t="s">
         <v>138</v>
       </c>
     </row>
@@ -4970,7 +4973,7 @@
       <c r="H104" s="9">
         <v>28</v>
       </c>
-      <c r="I104" s="15" t="s">
+      <c r="I104" s="16" t="s">
         <v>139</v>
       </c>
     </row>
@@ -4999,7 +5002,7 @@
       <c r="H105" s="5">
         <v>29</v>
       </c>
-      <c r="I105" s="15" t="s">
+      <c r="I105" s="16" t="s">
         <v>141</v>
       </c>
     </row>
@@ -5028,7 +5031,7 @@
       <c r="H106" s="5">
         <v>29</v>
       </c>
-      <c r="I106" s="15" t="s">
+      <c r="I106" s="16" t="s">
         <v>142</v>
       </c>
     </row>
@@ -5057,7 +5060,7 @@
       <c r="H107" s="5">
         <v>29</v>
       </c>
-      <c r="I107" s="15" t="s">
+      <c r="I107" s="16" t="s">
         <v>143</v>
       </c>
     </row>
@@ -5086,7 +5089,7 @@
       <c r="H108" s="5">
         <v>30</v>
       </c>
-      <c r="I108" s="15" t="s">
+      <c r="I108" s="16" t="s">
         <v>145</v>
       </c>
     </row>
@@ -5115,7 +5118,7 @@
       <c r="H109" s="5">
         <v>30</v>
       </c>
-      <c r="I109" s="15" t="s">
+      <c r="I109" s="16" t="s">
         <v>146</v>
       </c>
     </row>
@@ -5144,7 +5147,7 @@
       <c r="H110" s="5">
         <v>30</v>
       </c>
-      <c r="I110" s="15" t="s">
+      <c r="I110" s="16" t="s">
         <v>147</v>
       </c>
     </row>
@@ -5173,7 +5176,7 @@
       <c r="H111" s="5">
         <v>30</v>
       </c>
-      <c r="I111" s="15" t="s">
+      <c r="I111" s="16" t="s">
         <v>148</v>
       </c>
     </row>
@@ -5202,7 +5205,7 @@
       <c r="H112" s="5">
         <v>30</v>
       </c>
-      <c r="I112" s="15" t="s">
+      <c r="I112" s="16" t="s">
         <v>149</v>
       </c>
     </row>
@@ -5231,7 +5234,7 @@
       <c r="H113" s="5">
         <v>31</v>
       </c>
-      <c r="I113" s="15" t="s">
+      <c r="I113" s="16" t="s">
         <v>151</v>
       </c>
     </row>
@@ -5260,7 +5263,7 @@
       <c r="H114" s="5">
         <v>31</v>
       </c>
-      <c r="I114" s="15" t="s">
+      <c r="I114" s="16" t="s">
         <v>152</v>
       </c>
     </row>
@@ -5289,7 +5292,7 @@
       <c r="H115" s="5">
         <v>31</v>
       </c>
-      <c r="I115" s="15" t="s">
+      <c r="I115" s="16" t="s">
         <v>153</v>
       </c>
     </row>
@@ -5318,7 +5321,7 @@
       <c r="H116" s="5">
         <v>31</v>
       </c>
-      <c r="I116" s="15" t="s">
+      <c r="I116" s="16" t="s">
         <v>154</v>
       </c>
     </row>
@@ -5347,7 +5350,7 @@
       <c r="H117" s="5">
         <v>32</v>
       </c>
-      <c r="I117" s="15" t="s">
+      <c r="I117" s="16" t="s">
         <v>156</v>
       </c>
     </row>
@@ -5376,7 +5379,7 @@
       <c r="H118" s="5">
         <v>32</v>
       </c>
-      <c r="I118" s="15" t="s">
+      <c r="I118" s="16" t="s">
         <v>157</v>
       </c>
     </row>
@@ -5405,7 +5408,7 @@
       <c r="H119" s="5">
         <v>32</v>
       </c>
-      <c r="I119" s="15" t="s">
+      <c r="I119" s="16" t="s">
         <v>158</v>
       </c>
     </row>
@@ -5434,7 +5437,7 @@
       <c r="H120" s="5">
         <v>33</v>
       </c>
-      <c r="I120" s="15" t="s">
+      <c r="I120" s="16" t="s">
         <v>160</v>
       </c>
     </row>
@@ -5463,7 +5466,7 @@
       <c r="H121" s="5">
         <v>33</v>
       </c>
-      <c r="I121" s="15" t="s">
+      <c r="I121" s="16" t="s">
         <v>161</v>
       </c>
     </row>
@@ -5492,7 +5495,7 @@
       <c r="H122" s="5">
         <v>33</v>
       </c>
-      <c r="I122" s="15" t="s">
+      <c r="I122" s="16" t="s">
         <v>162</v>
       </c>
     </row>
@@ -5521,7 +5524,7 @@
       <c r="H123" s="5">
         <v>33</v>
       </c>
-      <c r="I123" s="15" t="s">
+      <c r="I123" s="16" t="s">
         <v>163</v>
       </c>
     </row>
@@ -5550,7 +5553,7 @@
       <c r="H124" s="5">
         <v>34</v>
       </c>
-      <c r="I124" s="15" t="s">
+      <c r="I124" s="16" t="s">
         <v>165</v>
       </c>
     </row>
@@ -5579,7 +5582,7 @@
       <c r="H125" s="5">
         <v>34</v>
       </c>
-      <c r="I125" s="15" t="s">
+      <c r="I125" s="16" t="s">
         <v>166</v>
       </c>
     </row>
@@ -5608,7 +5611,7 @@
       <c r="H126" s="5">
         <v>34</v>
       </c>
-      <c r="I126" s="15" t="s">
+      <c r="I126" s="16" t="s">
         <v>167</v>
       </c>
     </row>
@@ -5637,7 +5640,7 @@
       <c r="H127" s="5">
         <v>34</v>
       </c>
-      <c r="I127" s="15" t="s">
+      <c r="I127" s="16" t="s">
         <v>168</v>
       </c>
     </row>
@@ -5666,7 +5669,7 @@
       <c r="H128" s="5">
         <v>35</v>
       </c>
-      <c r="I128" s="15" t="s">
+      <c r="I128" s="16" t="s">
         <v>170</v>
       </c>
     </row>
@@ -5695,7 +5698,7 @@
       <c r="H129" s="5">
         <v>35</v>
       </c>
-      <c r="I129" s="15" t="s">
+      <c r="I129" s="16" t="s">
         <v>171</v>
       </c>
     </row>
@@ -5724,7 +5727,7 @@
       <c r="H130" s="5">
         <v>35</v>
       </c>
-      <c r="I130" s="15" t="s">
+      <c r="I130" s="16" t="s">
         <v>172</v>
       </c>
     </row>
@@ -5753,7 +5756,7 @@
       <c r="H131" s="5">
         <v>35</v>
       </c>
-      <c r="I131" s="15" t="s">
+      <c r="I131" s="16" t="s">
         <v>173</v>
       </c>
     </row>
@@ -5782,7 +5785,7 @@
       <c r="H132" s="5">
         <v>35</v>
       </c>
-      <c r="I132" s="15" t="s">
+      <c r="I132" s="16" t="s">
         <v>174</v>
       </c>
     </row>
@@ -5811,7 +5814,7 @@
       <c r="H133" s="7">
         <v>36</v>
       </c>
-      <c r="I133" s="15" t="s">
+      <c r="I133" s="16" t="s">
         <v>176</v>
       </c>
     </row>
@@ -5840,7 +5843,7 @@
       <c r="H134" s="7">
         <v>36</v>
       </c>
-      <c r="I134" s="15" t="s">
+      <c r="I134" s="16" t="s">
         <v>177</v>
       </c>
     </row>
@@ -5869,7 +5872,7 @@
       <c r="H135" s="7">
         <v>36</v>
       </c>
-      <c r="I135" s="15" t="s">
+      <c r="I135" s="16" t="s">
         <v>178</v>
       </c>
     </row>
@@ -5898,7 +5901,7 @@
       <c r="H136" s="7">
         <v>36</v>
       </c>
-      <c r="I136" s="15" t="s">
+      <c r="I136" s="16" t="s">
         <v>179</v>
       </c>
     </row>
@@ -5927,7 +5930,7 @@
       <c r="H137" s="7">
         <v>36</v>
       </c>
-      <c r="I137" s="15" t="s">
+      <c r="I137" s="16" t="s">
         <v>180</v>
       </c>
     </row>
@@ -5956,7 +5959,7 @@
       <c r="H138" s="7">
         <v>36</v>
       </c>
-      <c r="I138" s="15" t="s">
+      <c r="I138" s="16" t="s">
         <v>181</v>
       </c>
     </row>
@@ -5985,7 +5988,7 @@
       <c r="H139" s="5">
         <v>37</v>
       </c>
-      <c r="I139" s="15" t="s">
+      <c r="I139" s="16" t="s">
         <v>183</v>
       </c>
     </row>
@@ -6014,7 +6017,7 @@
       <c r="H140" s="5">
         <v>37</v>
       </c>
-      <c r="I140" s="15" t="s">
+      <c r="I140" s="16" t="s">
         <v>184</v>
       </c>
     </row>
@@ -6043,7 +6046,7 @@
       <c r="H141" s="5">
         <v>37</v>
       </c>
-      <c r="I141" s="15" t="s">
+      <c r="I141" s="16" t="s">
         <v>185</v>
       </c>
     </row>
@@ -6072,7 +6075,7 @@
       <c r="H142" s="5">
         <v>37</v>
       </c>
-      <c r="I142" s="15" t="s">
+      <c r="I142" s="16" t="s">
         <v>186</v>
       </c>
     </row>
@@ -6101,7 +6104,7 @@
       <c r="H143" s="5">
         <v>38</v>
       </c>
-      <c r="I143" s="15" t="s">
+      <c r="I143" s="16" t="s">
         <v>188</v>
       </c>
     </row>
@@ -6130,7 +6133,7 @@
       <c r="H144" s="5">
         <v>38</v>
       </c>
-      <c r="I144" s="15" t="s">
+      <c r="I144" s="16" t="s">
         <v>189</v>
       </c>
     </row>
@@ -6159,7 +6162,7 @@
       <c r="H145" s="5">
         <v>38</v>
       </c>
-      <c r="I145" s="15" t="s">
+      <c r="I145" s="16" t="s">
         <v>190</v>
       </c>
     </row>
@@ -6188,7 +6191,7 @@
       <c r="H146" s="5">
         <v>38</v>
       </c>
-      <c r="I146" s="15" t="s">
+      <c r="I146" s="16" t="s">
         <v>191</v>
       </c>
     </row>
@@ -6217,7 +6220,7 @@
       <c r="H147" s="5">
         <v>39</v>
       </c>
-      <c r="I147" s="15" t="s">
+      <c r="I147" s="16" t="s">
         <v>193</v>
       </c>
     </row>
@@ -6246,7 +6249,7 @@
       <c r="H148" s="5">
         <v>39</v>
       </c>
-      <c r="I148" s="15" t="s">
+      <c r="I148" s="16" t="s">
         <v>194</v>
       </c>
     </row>
@@ -6275,7 +6278,7 @@
       <c r="H149" s="5">
         <v>39</v>
       </c>
-      <c r="I149" s="15" t="s">
+      <c r="I149" s="16" t="s">
         <v>195</v>
       </c>
     </row>
@@ -6304,7 +6307,7 @@
       <c r="H150" s="5">
         <v>39</v>
       </c>
-      <c r="I150" s="15" t="s">
+      <c r="I150" s="16" t="s">
         <v>196</v>
       </c>
     </row>
@@ -6333,7 +6336,7 @@
       <c r="H151" s="5">
         <v>40</v>
       </c>
-      <c r="I151" s="15" t="s">
+      <c r="I151" s="16" t="s">
         <v>198</v>
       </c>
     </row>
@@ -6362,7 +6365,7 @@
       <c r="H152" s="5">
         <v>40</v>
       </c>
-      <c r="I152" s="15" t="s">
+      <c r="I152" s="16" t="s">
         <v>199</v>
       </c>
     </row>
@@ -6391,7 +6394,7 @@
       <c r="H153" s="5">
         <v>40</v>
       </c>
-      <c r="I153" s="15" t="s">
+      <c r="I153" s="16" t="s">
         <v>200</v>
       </c>
     </row>
@@ -6420,7 +6423,7 @@
       <c r="H154" s="5">
         <v>40</v>
       </c>
-      <c r="I154" s="15" t="s">
+      <c r="I154" s="16" t="s">
         <v>201</v>
       </c>
     </row>
@@ -6449,7 +6452,7 @@
       <c r="H155" s="5">
         <v>41</v>
       </c>
-      <c r="I155" s="15" t="s">
+      <c r="I155" s="16" t="s">
         <v>203</v>
       </c>
     </row>
@@ -6478,7 +6481,7 @@
       <c r="H156" s="5">
         <v>41</v>
       </c>
-      <c r="I156" s="15" t="s">
+      <c r="I156" s="16" t="s">
         <v>204</v>
       </c>
     </row>
@@ -6507,7 +6510,7 @@
       <c r="H157" s="5">
         <v>41</v>
       </c>
-      <c r="I157" s="15" t="s">
+      <c r="I157" s="16" t="s">
         <v>205</v>
       </c>
     </row>
@@ -6536,7 +6539,7 @@
       <c r="H158" s="5">
         <v>41</v>
       </c>
-      <c r="I158" s="15" t="s">
+      <c r="I158" s="16" t="s">
         <v>206</v>
       </c>
     </row>
@@ -6565,7 +6568,7 @@
       <c r="H159" s="5">
         <v>42</v>
       </c>
-      <c r="I159" s="15" t="s">
+      <c r="I159" s="16" t="s">
         <v>208</v>
       </c>
     </row>
@@ -6594,7 +6597,7 @@
       <c r="H160" s="5">
         <v>42</v>
       </c>
-      <c r="I160" s="15" t="s">
+      <c r="I160" s="16" t="s">
         <v>209</v>
       </c>
     </row>
@@ -6623,7 +6626,7 @@
       <c r="H161" s="5">
         <v>42</v>
       </c>
-      <c r="I161" s="15" t="s">
+      <c r="I161" s="16" t="s">
         <v>210</v>
       </c>
     </row>
@@ -6652,7 +6655,7 @@
       <c r="H162" s="5">
         <v>42</v>
       </c>
-      <c r="I162" s="15" t="s">
+      <c r="I162" s="16" t="s">
         <v>211</v>
       </c>
     </row>
@@ -6681,7 +6684,7 @@
       <c r="H163" s="5">
         <v>42</v>
       </c>
-      <c r="I163" s="15" t="s">
+      <c r="I163" s="16" t="s">
         <v>212</v>
       </c>
     </row>
@@ -6710,7 +6713,7 @@
       <c r="H164" s="5">
         <v>43</v>
       </c>
-      <c r="I164" s="15" t="s">
+      <c r="I164" s="16" t="s">
         <v>214</v>
       </c>
     </row>
@@ -6739,7 +6742,7 @@
       <c r="H165" s="5">
         <v>43</v>
       </c>
-      <c r="I165" s="15" t="s">
+      <c r="I165" s="16" t="s">
         <v>215</v>
       </c>
     </row>
@@ -6768,7 +6771,7 @@
       <c r="H166" s="5">
         <v>43</v>
       </c>
-      <c r="I166" s="15" t="s">
+      <c r="I166" s="16" t="s">
         <v>216</v>
       </c>
     </row>
@@ -6797,7 +6800,7 @@
       <c r="H167" s="5">
         <v>43</v>
       </c>
-      <c r="I167" s="15" t="s">
+      <c r="I167" s="16" t="s">
         <v>217</v>
       </c>
     </row>
@@ -6826,7 +6829,7 @@
       <c r="H168" s="5">
         <v>44</v>
       </c>
-      <c r="I168" s="15" t="s">
+      <c r="I168" s="16" t="s">
         <v>219</v>
       </c>
     </row>
@@ -6855,7 +6858,7 @@
       <c r="H169" s="5">
         <v>44</v>
       </c>
-      <c r="I169" s="15" t="s">
+      <c r="I169" s="16" t="s">
         <v>220</v>
       </c>
     </row>
@@ -6884,7 +6887,7 @@
       <c r="H170" s="5">
         <v>44</v>
       </c>
-      <c r="I170" s="15" t="s">
+      <c r="I170" s="16" t="s">
         <v>221</v>
       </c>
     </row>
@@ -6913,7 +6916,7 @@
       <c r="H171" s="5">
         <v>44</v>
       </c>
-      <c r="I171" s="15" t="s">
+      <c r="I171" s="16" t="s">
         <v>222</v>
       </c>
     </row>
@@ -6942,7 +6945,7 @@
       <c r="H172" s="5">
         <v>45</v>
       </c>
-      <c r="I172" s="15" t="s">
+      <c r="I172" s="16" t="s">
         <v>224</v>
       </c>
     </row>
@@ -6971,7 +6974,7 @@
       <c r="H173" s="5">
         <v>45</v>
       </c>
-      <c r="I173" s="15" t="s">
+      <c r="I173" s="16" t="s">
         <v>225</v>
       </c>
     </row>
@@ -7000,7 +7003,7 @@
       <c r="H174" s="5">
         <v>45</v>
       </c>
-      <c r="I174" s="15" t="s">
+      <c r="I174" s="16" t="s">
         <v>226</v>
       </c>
     </row>
@@ -7029,7 +7032,7 @@
       <c r="H175" s="5">
         <v>45</v>
       </c>
-      <c r="I175" s="15" t="s">
+      <c r="I175" s="16" t="s">
         <v>227</v>
       </c>
     </row>
@@ -7058,7 +7061,7 @@
       <c r="H176" s="5">
         <v>46</v>
       </c>
-      <c r="I176" s="15" t="s">
+      <c r="I176" s="16" t="s">
         <v>229</v>
       </c>
     </row>
@@ -7087,7 +7090,7 @@
       <c r="H177" s="5">
         <v>46</v>
       </c>
-      <c r="I177" s="15" t="s">
+      <c r="I177" s="16" t="s">
         <v>230</v>
       </c>
     </row>
@@ -7116,7 +7119,7 @@
       <c r="H178" s="5">
         <v>46</v>
       </c>
-      <c r="I178" s="15" t="s">
+      <c r="I178" s="16" t="s">
         <v>231</v>
       </c>
     </row>
@@ -7145,7 +7148,7 @@
       <c r="H179" s="5">
         <v>47</v>
       </c>
-      <c r="I179" s="15" t="s">
+      <c r="I179" s="16" t="s">
         <v>233</v>
       </c>
     </row>
@@ -7174,7 +7177,7 @@
       <c r="H180" s="5">
         <v>47</v>
       </c>
-      <c r="I180" s="15" t="s">
+      <c r="I180" s="16" t="s">
         <v>234</v>
       </c>
     </row>
@@ -7203,7 +7206,7 @@
       <c r="H181" s="5">
         <v>47</v>
       </c>
-      <c r="I181" s="15" t="s">
+      <c r="I181" s="16" t="s">
         <v>235</v>
       </c>
     </row>
@@ -7232,7 +7235,7 @@
       <c r="H182" s="5">
         <v>48</v>
       </c>
-      <c r="I182" s="15" t="s">
+      <c r="I182" s="16" t="s">
         <v>237</v>
       </c>
     </row>
@@ -7261,7 +7264,7 @@
       <c r="H183" s="5">
         <v>48</v>
       </c>
-      <c r="I183" s="15" t="s">
+      <c r="I183" s="16" t="s">
         <v>238</v>
       </c>
     </row>
@@ -7290,7 +7293,7 @@
       <c r="H184" s="5">
         <v>48</v>
       </c>
-      <c r="I184" s="15" t="s">
+      <c r="I184" s="16" t="s">
         <v>239</v>
       </c>
     </row>
@@ -7319,7 +7322,7 @@
       <c r="H185" s="5">
         <v>49</v>
       </c>
-      <c r="I185" s="15" t="s">
+      <c r="I185" s="16" t="s">
         <v>241</v>
       </c>
     </row>
@@ -7348,7 +7351,7 @@
       <c r="H186" s="5">
         <v>49</v>
       </c>
-      <c r="I186" s="15" t="s">
+      <c r="I186" s="16" t="s">
         <v>242</v>
       </c>
     </row>
@@ -7377,7 +7380,7 @@
       <c r="H187" s="5">
         <v>49</v>
       </c>
-      <c r="I187" s="15" t="s">
+      <c r="I187" s="16" t="s">
         <v>243</v>
       </c>
     </row>
@@ -7406,7 +7409,7 @@
       <c r="H188" s="5">
         <v>50</v>
       </c>
-      <c r="I188" s="15" t="s">
+      <c r="I188" s="16" t="s">
         <v>245</v>
       </c>
     </row>
@@ -7435,7 +7438,7 @@
       <c r="H189" s="5">
         <v>49</v>
       </c>
-      <c r="I189" s="15" t="s">
+      <c r="I189" s="16" t="s">
         <v>246</v>
       </c>
     </row>
@@ -7464,7 +7467,7 @@
       <c r="H190" s="5">
         <v>49</v>
       </c>
-      <c r="I190" s="15" t="s">
+      <c r="I190" s="16" t="s">
         <v>247</v>
       </c>
     </row>
@@ -7493,7 +7496,7 @@
       <c r="H191" s="5">
         <v>51</v>
       </c>
-      <c r="I191" s="15" t="s">
+      <c r="I191" s="16" t="s">
         <v>249</v>
       </c>
     </row>
@@ -7522,7 +7525,7 @@
       <c r="H192" s="5">
         <v>51</v>
       </c>
-      <c r="I192" s="15" t="s">
+      <c r="I192" s="16" t="s">
         <v>250</v>
       </c>
     </row>
@@ -7551,7 +7554,7 @@
       <c r="H193" s="5">
         <v>51</v>
       </c>
-      <c r="I193" s="15" t="s">
+      <c r="I193" s="16" t="s">
         <v>251</v>
       </c>
     </row>
@@ -7580,7 +7583,7 @@
       <c r="H194" s="5">
         <v>52</v>
       </c>
-      <c r="I194" s="15" t="s">
+      <c r="I194" s="16" t="s">
         <v>253</v>
       </c>
     </row>
@@ -7609,7 +7612,7 @@
       <c r="H195" s="5">
         <v>52</v>
       </c>
-      <c r="I195" s="15" t="s">
+      <c r="I195" s="16" t="s">
         <v>254</v>
       </c>
     </row>
@@ -7638,7 +7641,7 @@
       <c r="H196" s="5">
         <v>52</v>
       </c>
-      <c r="I196" s="15" t="s">
+      <c r="I196" s="16" t="s">
         <v>255</v>
       </c>
     </row>
@@ -7667,7 +7670,7 @@
       <c r="H197" s="5">
         <v>53</v>
       </c>
-      <c r="I197" s="15" t="s">
+      <c r="I197" s="16" t="s">
         <v>257</v>
       </c>
     </row>
@@ -7696,7 +7699,7 @@
       <c r="H198" s="5">
         <v>53</v>
       </c>
-      <c r="I198" s="15" t="s">
+      <c r="I198" s="16" t="s">
         <v>258</v>
       </c>
     </row>
@@ -7725,7 +7728,7 @@
       <c r="H199" s="5">
         <v>53</v>
       </c>
-      <c r="I199" s="15" t="s">
+      <c r="I199" s="16" t="s">
         <v>259</v>
       </c>
     </row>
@@ -7754,7 +7757,7 @@
       <c r="H200" s="5">
         <v>54</v>
       </c>
-      <c r="I200" s="15" t="s">
+      <c r="I200" s="16" t="s">
         <v>261</v>
       </c>
     </row>
@@ -7783,7 +7786,7 @@
       <c r="H201" s="5">
         <v>54</v>
       </c>
-      <c r="I201" s="15" t="s">
+      <c r="I201" s="16" t="s">
         <v>262</v>
       </c>
     </row>
@@ -7812,7 +7815,7 @@
       <c r="H202" s="5">
         <v>54</v>
       </c>
-      <c r="I202" s="15" t="s">
+      <c r="I202" s="16" t="s">
         <v>263</v>
       </c>
     </row>
@@ -7841,7 +7844,7 @@
       <c r="H203" s="5">
         <v>55</v>
       </c>
-      <c r="I203" s="15" t="s">
+      <c r="I203" s="16" t="s">
         <v>265</v>
       </c>
     </row>
@@ -7870,7 +7873,7 @@
       <c r="H204" s="5">
         <v>55</v>
       </c>
-      <c r="I204" s="15" t="s">
+      <c r="I204" s="16" t="s">
         <v>266</v>
       </c>
     </row>
@@ -7899,7 +7902,7 @@
       <c r="H205" s="5">
         <v>55</v>
       </c>
-      <c r="I205" s="15" t="s">
+      <c r="I205" s="16" t="s">
         <v>267</v>
       </c>
     </row>
@@ -7928,7 +7931,7 @@
       <c r="H206" s="5">
         <v>56</v>
       </c>
-      <c r="I206" s="15" t="s">
+      <c r="I206" s="16" t="s">
         <v>269</v>
       </c>
     </row>
@@ -7957,7 +7960,7 @@
       <c r="H207" s="5">
         <v>56</v>
       </c>
-      <c r="I207" s="15" t="s">
+      <c r="I207" s="16" t="s">
         <v>270</v>
       </c>
     </row>
@@ -7986,7 +7989,7 @@
       <c r="H208" s="5">
         <v>56</v>
       </c>
-      <c r="I208" s="15" t="s">
+      <c r="I208" s="16" t="s">
         <v>271</v>
       </c>
     </row>
@@ -8015,7 +8018,7 @@
       <c r="H209" s="5">
         <v>57</v>
       </c>
-      <c r="I209" s="15" t="s">
+      <c r="I209" s="16" t="s">
         <v>273</v>
       </c>
     </row>
@@ -8044,7 +8047,7 @@
       <c r="H210" s="5">
         <v>57</v>
       </c>
-      <c r="I210" s="15" t="s">
+      <c r="I210" s="16" t="s">
         <v>274</v>
       </c>
     </row>
@@ -8073,7 +8076,7 @@
       <c r="H211" s="5">
         <v>57</v>
       </c>
-      <c r="I211" s="15" t="s">
+      <c r="I211" s="16" t="s">
         <v>275</v>
       </c>
     </row>
@@ -8102,7 +8105,7 @@
       <c r="H212" s="5">
         <v>57</v>
       </c>
-      <c r="I212" s="15" t="s">
+      <c r="I212" s="16" t="s">
         <v>276</v>
       </c>
     </row>
@@ -8131,7 +8134,7 @@
       <c r="H213" s="5">
         <v>58</v>
       </c>
-      <c r="I213" s="15" t="s">
+      <c r="I213" s="16" t="s">
         <v>278</v>
       </c>
     </row>
@@ -8160,7 +8163,7 @@
       <c r="H214" s="5">
         <v>58</v>
       </c>
-      <c r="I214" s="15" t="s">
+      <c r="I214" s="16" t="s">
         <v>279</v>
       </c>
     </row>
@@ -8189,7 +8192,7 @@
       <c r="H215" s="5">
         <v>58</v>
       </c>
-      <c r="I215" s="15" t="s">
+      <c r="I215" s="16" t="s">
         <v>280</v>
       </c>
     </row>
@@ -8218,7 +8221,7 @@
       <c r="H216" s="5">
         <v>58</v>
       </c>
-      <c r="I216" s="15" t="s">
+      <c r="I216" s="16" t="s">
         <v>281</v>
       </c>
     </row>
@@ -8247,7 +8250,7 @@
       <c r="H217" s="5">
         <v>59</v>
       </c>
-      <c r="I217" s="15" t="s">
+      <c r="I217" s="16" t="s">
         <v>283</v>
       </c>
     </row>
@@ -8276,7 +8279,7 @@
       <c r="H218" s="5">
         <v>59</v>
       </c>
-      <c r="I218" s="15" t="s">
+      <c r="I218" s="16" t="s">
         <v>284</v>
       </c>
     </row>
@@ -8305,7 +8308,7 @@
       <c r="H219" s="5">
         <v>59</v>
       </c>
-      <c r="I219" s="15" t="s">
+      <c r="I219" s="16" t="s">
         <v>285</v>
       </c>
     </row>
@@ -8334,7 +8337,7 @@
       <c r="H220" s="5">
         <v>60</v>
       </c>
-      <c r="I220" s="15" t="s">
+      <c r="I220" s="16" t="s">
         <v>287</v>
       </c>
     </row>
@@ -8363,7 +8366,7 @@
       <c r="H221" s="5">
         <v>60</v>
       </c>
-      <c r="I221" s="15" t="s">
+      <c r="I221" s="16" t="s">
         <v>288</v>
       </c>
     </row>
@@ -8392,7 +8395,7 @@
       <c r="H222" s="5">
         <v>60</v>
       </c>
-      <c r="I222" s="15" t="s">
+      <c r="I222" s="16" t="s">
         <v>289</v>
       </c>
     </row>
@@ -8421,7 +8424,7 @@
       <c r="H223" s="5">
         <v>61</v>
       </c>
-      <c r="I223" s="15" t="s">
+      <c r="I223" s="16" t="s">
         <v>291</v>
       </c>
     </row>
@@ -8450,7 +8453,7 @@
       <c r="H224" s="5">
         <v>61</v>
       </c>
-      <c r="I224" s="15" t="s">
+      <c r="I224" s="16" t="s">
         <v>292</v>
       </c>
     </row>
@@ -8479,7 +8482,7 @@
       <c r="H225" s="5">
         <v>61</v>
       </c>
-      <c r="I225" s="15" t="s">
+      <c r="I225" s="16" t="s">
         <v>293</v>
       </c>
     </row>
@@ -8508,7 +8511,7 @@
       <c r="H226" s="5">
         <v>62</v>
       </c>
-      <c r="I226" s="15" t="s">
+      <c r="I226" s="16" t="s">
         <v>295</v>
       </c>
     </row>
@@ -8537,7 +8540,7 @@
       <c r="H227" s="5">
         <v>62</v>
       </c>
-      <c r="I227" s="15" t="s">
+      <c r="I227" s="16" t="s">
         <v>296</v>
       </c>
     </row>
@@ -8566,7 +8569,7 @@
       <c r="H228" s="5">
         <v>62</v>
       </c>
-      <c r="I228" s="15" t="s">
+      <c r="I228" s="16" t="s">
         <v>297</v>
       </c>
     </row>
@@ -8595,7 +8598,7 @@
       <c r="H229" s="5">
         <v>63</v>
       </c>
-      <c r="I229" s="15" t="s">
+      <c r="I229" s="16" t="s">
         <v>299</v>
       </c>
     </row>
@@ -8624,7 +8627,7 @@
       <c r="H230" s="5">
         <v>63</v>
       </c>
-      <c r="I230" s="15" t="s">
+      <c r="I230" s="16" t="s">
         <v>300</v>
       </c>
     </row>
@@ -8653,7 +8656,7 @@
       <c r="H231" s="5">
         <v>64</v>
       </c>
-      <c r="I231" s="15" t="s">
+      <c r="I231" s="16" t="s">
         <v>302</v>
       </c>
     </row>
@@ -8682,7 +8685,7 @@
       <c r="H232" s="5">
         <v>64</v>
       </c>
-      <c r="I232" s="15" t="s">
+      <c r="I232" s="16" t="s">
         <v>303</v>
       </c>
     </row>
@@ -8711,7 +8714,7 @@
       <c r="H233" s="5">
         <v>64</v>
       </c>
-      <c r="I233" s="15" t="s">
+      <c r="I233" s="16" t="s">
         <v>304</v>
       </c>
     </row>
@@ -8740,7 +8743,7 @@
       <c r="H234" s="5">
         <v>65</v>
       </c>
-      <c r="I234" s="15" t="s">
+      <c r="I234" s="16" t="s">
         <v>306</v>
       </c>
     </row>
@@ -8769,7 +8772,7 @@
       <c r="H235" s="5">
         <v>65</v>
       </c>
-      <c r="I235" s="15" t="s">
+      <c r="I235" s="16" t="s">
         <v>307</v>
       </c>
     </row>
@@ -8798,7 +8801,7 @@
       <c r="H236" s="5">
         <v>65</v>
       </c>
-      <c r="I236" s="15" t="s">
+      <c r="I236" s="16" t="s">
         <v>308</v>
       </c>
     </row>
@@ -8827,7 +8830,7 @@
       <c r="H237" s="5">
         <v>66</v>
       </c>
-      <c r="I237" s="15" t="s">
+      <c r="I237" s="16" t="s">
         <v>310</v>
       </c>
     </row>
@@ -8856,7 +8859,7 @@
       <c r="H238" s="5">
         <v>66</v>
       </c>
-      <c r="I238" s="15" t="s">
+      <c r="I238" s="16" t="s">
         <v>311</v>
       </c>
     </row>
@@ -8885,7 +8888,7 @@
       <c r="H239" s="5">
         <v>66</v>
       </c>
-      <c r="I239" s="15" t="s">
+      <c r="I239" s="16" t="s">
         <v>312</v>
       </c>
       <c r="J239" s="1"/>
@@ -8916,7 +8919,7 @@
       <c r="H240" s="5">
         <v>67</v>
       </c>
-      <c r="I240" s="15" t="s">
+      <c r="I240" s="16" t="s">
         <v>314</v>
       </c>
     </row>
@@ -8945,7 +8948,7 @@
       <c r="H241" s="5">
         <v>67</v>
       </c>
-      <c r="I241" s="15" t="s">
+      <c r="I241" s="16" t="s">
         <v>315</v>
       </c>
     </row>
@@ -8974,7 +8977,7 @@
       <c r="H242" s="5">
         <v>67</v>
       </c>
-      <c r="I242" s="15" t="s">
+      <c r="I242" s="16" t="s">
         <v>316</v>
       </c>
     </row>
@@ -9003,7 +9006,7 @@
       <c r="H243" s="5">
         <v>67</v>
       </c>
-      <c r="I243" s="15" t="s">
+      <c r="I243" s="16" t="s">
         <v>317</v>
       </c>
     </row>
@@ -9032,7 +9035,7 @@
       <c r="H244" s="5">
         <v>68</v>
       </c>
-      <c r="I244" s="15" t="s">
+      <c r="I244" s="16" t="s">
         <v>319</v>
       </c>
     </row>
@@ -9061,7 +9064,7 @@
       <c r="H245" s="5">
         <v>68</v>
       </c>
-      <c r="I245" s="15" t="s">
+      <c r="I245" s="16" t="s">
         <v>320</v>
       </c>
     </row>
@@ -9090,7 +9093,7 @@
       <c r="H246" s="5">
         <v>68</v>
       </c>
-      <c r="I246" s="15" t="s">
+      <c r="I246" s="16" t="s">
         <v>321</v>
       </c>
     </row>
@@ -9119,7 +9122,7 @@
       <c r="H247" s="5">
         <v>68</v>
       </c>
-      <c r="I247" s="15" t="s">
+      <c r="I247" s="16" t="s">
         <v>322</v>
       </c>
     </row>
@@ -9148,7 +9151,7 @@
       <c r="H248" s="5">
         <v>69</v>
       </c>
-      <c r="I248" s="15" t="s">
+      <c r="I248" s="16" t="s">
         <v>324</v>
       </c>
     </row>
@@ -9177,7 +9180,7 @@
       <c r="H249" s="5">
         <v>69</v>
       </c>
-      <c r="I249" s="15" t="s">
+      <c r="I249" s="16" t="s">
         <v>325</v>
       </c>
     </row>
@@ -9206,7 +9209,7 @@
       <c r="H250" s="5">
         <v>69</v>
       </c>
-      <c r="I250" s="15" t="s">
+      <c r="I250" s="16" t="s">
         <v>326</v>
       </c>
     </row>
@@ -9235,7 +9238,7 @@
       <c r="H251" s="5">
         <v>70</v>
       </c>
-      <c r="I251" s="15" t="s">
+      <c r="I251" s="16" t="s">
         <v>328</v>
       </c>
     </row>
@@ -9264,7 +9267,7 @@
       <c r="H252" s="5">
         <v>70</v>
       </c>
-      <c r="I252" s="15" t="s">
+      <c r="I252" s="16" t="s">
         <v>329</v>
       </c>
     </row>
@@ -9293,7 +9296,7 @@
       <c r="H253" s="5">
         <v>70</v>
       </c>
-      <c r="I253" s="15" t="s">
+      <c r="I253" s="16" t="s">
         <v>330</v>
       </c>
     </row>
@@ -9322,7 +9325,7 @@
       <c r="H254" s="5">
         <v>70</v>
       </c>
-      <c r="I254" s="15" t="s">
+      <c r="I254" s="16" t="s">
         <v>331</v>
       </c>
     </row>
@@ -9351,7 +9354,7 @@
       <c r="H255" s="5">
         <v>71</v>
       </c>
-      <c r="I255" s="15" t="s">
+      <c r="I255" s="16" t="s">
         <v>333</v>
       </c>
     </row>
@@ -9380,7 +9383,7 @@
       <c r="H256" s="5">
         <v>71</v>
       </c>
-      <c r="I256" s="15" t="s">
+      <c r="I256" s="16" t="s">
         <v>334</v>
       </c>
     </row>
@@ -9409,7 +9412,7 @@
       <c r="H257" s="5">
         <v>71</v>
       </c>
-      <c r="I257" s="15" t="s">
+      <c r="I257" s="16" t="s">
         <v>335</v>
       </c>
     </row>
@@ -9438,7 +9441,7 @@
       <c r="H258" s="5">
         <v>72</v>
       </c>
-      <c r="I258" s="15" t="s">
+      <c r="I258" s="16" t="s">
         <v>337</v>
       </c>
     </row>
@@ -9467,7 +9470,7 @@
       <c r="H259" s="5">
         <v>72</v>
       </c>
-      <c r="I259" s="15" t="s">
+      <c r="I259" s="16" t="s">
         <v>338</v>
       </c>
     </row>
@@ -9496,7 +9499,7 @@
       <c r="H260" s="5">
         <v>72</v>
       </c>
-      <c r="I260" s="15" t="s">
+      <c r="I260" s="16" t="s">
         <v>339</v>
       </c>
     </row>
@@ -9525,7 +9528,7 @@
       <c r="H261" s="5">
         <v>73</v>
       </c>
-      <c r="I261" s="15" t="s">
+      <c r="I261" s="16" t="s">
         <v>341</v>
       </c>
     </row>
@@ -9554,7 +9557,7 @@
       <c r="H262" s="5">
         <v>73</v>
       </c>
-      <c r="I262" s="15" t="s">
+      <c r="I262" s="16" t="s">
         <v>342</v>
       </c>
     </row>
@@ -9583,7 +9586,7 @@
       <c r="H263" s="5">
         <v>73</v>
       </c>
-      <c r="I263" s="15" t="s">
+      <c r="I263" s="16" t="s">
         <v>343</v>
       </c>
     </row>
@@ -9612,7 +9615,7 @@
       <c r="H264" s="5">
         <v>73</v>
       </c>
-      <c r="I264" s="15" t="s">
+      <c r="I264" s="16" t="s">
         <v>344</v>
       </c>
     </row>
@@ -9641,7 +9644,7 @@
       <c r="H265" s="5">
         <v>74</v>
       </c>
-      <c r="I265" s="15" t="s">
+      <c r="I265" s="16" t="s">
         <v>346</v>
       </c>
     </row>
@@ -9670,7 +9673,7 @@
       <c r="H266" s="5">
         <v>74</v>
       </c>
-      <c r="I266" s="15" t="s">
+      <c r="I266" s="16" t="s">
         <v>347</v>
       </c>
     </row>
@@ -9699,7 +9702,7 @@
       <c r="H267" s="5">
         <v>74</v>
       </c>
-      <c r="I267" s="15" t="s">
+      <c r="I267" s="16" t="s">
         <v>348</v>
       </c>
     </row>
@@ -9728,7 +9731,7 @@
       <c r="H268" s="5">
         <v>75</v>
       </c>
-      <c r="I268" s="15" t="s">
+      <c r="I268" s="16" t="s">
         <v>350</v>
       </c>
     </row>
@@ -9757,7 +9760,7 @@
       <c r="H269" s="5">
         <v>75</v>
       </c>
-      <c r="I269" s="15" t="s">
+      <c r="I269" s="16" t="s">
         <v>351</v>
       </c>
     </row>
@@ -9786,7 +9789,7 @@
       <c r="H270" s="5">
         <v>75</v>
       </c>
-      <c r="I270" s="15" t="s">
+      <c r="I270" s="16" t="s">
         <v>352</v>
       </c>
     </row>
@@ -9815,7 +9818,7 @@
       <c r="H271" s="5">
         <v>75</v>
       </c>
-      <c r="I271" s="15" t="s">
+      <c r="I271" s="16" t="s">
         <v>353</v>
       </c>
     </row>
@@ -9844,7 +9847,7 @@
       <c r="H272" s="5">
         <v>76</v>
       </c>
-      <c r="I272" s="15" t="s">
+      <c r="I272" s="16" t="s">
         <v>355</v>
       </c>
     </row>
@@ -9873,7 +9876,7 @@
       <c r="H273" s="5">
         <v>76</v>
       </c>
-      <c r="I273" s="15" t="s">
+      <c r="I273" s="16" t="s">
         <v>356</v>
       </c>
     </row>
@@ -9902,7 +9905,7 @@
       <c r="H274" s="5">
         <v>76</v>
       </c>
-      <c r="I274" s="15" t="s">
+      <c r="I274" s="16" t="s">
         <v>357</v>
       </c>
     </row>
@@ -9931,7 +9934,7 @@
       <c r="H275" s="5">
         <v>77</v>
       </c>
-      <c r="I275" s="15" t="s">
+      <c r="I275" s="16" t="s">
         <v>359</v>
       </c>
     </row>
@@ -9960,7 +9963,7 @@
       <c r="H276" s="5">
         <v>77</v>
       </c>
-      <c r="I276" s="15" t="s">
+      <c r="I276" s="16" t="s">
         <v>360</v>
       </c>
     </row>
@@ -9989,7 +9992,7 @@
       <c r="H277" s="5">
         <v>77</v>
       </c>
-      <c r="I277" s="15" t="s">
+      <c r="I277" s="16" t="s">
         <v>361</v>
       </c>
     </row>
@@ -10018,7 +10021,7 @@
       <c r="H278" s="5">
         <v>78</v>
       </c>
-      <c r="I278" s="15" t="s">
+      <c r="I278" s="16" t="s">
         <v>363</v>
       </c>
     </row>
@@ -10047,7 +10050,7 @@
       <c r="H279" s="5">
         <v>78</v>
       </c>
-      <c r="I279" s="15" t="s">
+      <c r="I279" s="16" t="s">
         <v>364</v>
       </c>
     </row>
@@ -10076,7 +10079,7 @@
       <c r="H280" s="5">
         <v>79</v>
       </c>
-      <c r="I280" s="15" t="s">
+      <c r="I280" s="16" t="s">
         <v>366</v>
       </c>
     </row>
@@ -10105,7 +10108,7 @@
       <c r="H281" s="5">
         <v>79</v>
       </c>
-      <c r="I281" s="15" t="s">
+      <c r="I281" s="16" t="s">
         <v>367</v>
       </c>
     </row>
@@ -10134,7 +10137,7 @@
       <c r="H282" s="5">
         <v>80</v>
       </c>
-      <c r="I282" s="15" t="s">
+      <c r="I282" s="16" t="s">
         <v>369</v>
       </c>
     </row>
@@ -10163,7 +10166,7 @@
       <c r="H283" s="5">
         <v>80</v>
       </c>
-      <c r="I283" s="15" t="s">
+      <c r="I283" s="16" t="s">
         <v>370</v>
       </c>
     </row>
@@ -10192,7 +10195,7 @@
       <c r="H284" s="5">
         <v>81</v>
       </c>
-      <c r="I284" s="15" t="s">
+      <c r="I284" s="16" t="s">
         <v>372</v>
       </c>
     </row>
@@ -10221,7 +10224,7 @@
       <c r="H285" s="5">
         <v>81</v>
       </c>
-      <c r="I285" s="15" t="s">
+      <c r="I285" s="16" t="s">
         <v>373</v>
       </c>
     </row>
@@ -10250,7 +10253,7 @@
       <c r="H286" s="5">
         <v>82</v>
       </c>
-      <c r="I286" s="15" t="s">
+      <c r="I286" s="16" t="s">
         <v>375</v>
       </c>
     </row>
@@ -10279,7 +10282,7 @@
       <c r="H287" s="5">
         <v>82</v>
       </c>
-      <c r="I287" s="15" t="s">
+      <c r="I287" s="16" t="s">
         <v>376</v>
       </c>
     </row>
@@ -10308,7 +10311,7 @@
       <c r="H288" s="5">
         <v>82</v>
       </c>
-      <c r="I288" s="15" t="s">
+      <c r="I288" s="16" t="s">
         <v>377</v>
       </c>
     </row>
@@ -10337,7 +10340,7 @@
       <c r="H289" s="5">
         <v>83</v>
       </c>
-      <c r="I289" s="15" t="s">
+      <c r="I289" s="16" t="s">
         <v>379</v>
       </c>
     </row>
@@ -10366,7 +10369,7 @@
       <c r="H290" s="5">
         <v>83</v>
       </c>
-      <c r="I290" s="15" t="s">
+      <c r="I290" s="16" t="s">
         <v>380</v>
       </c>
     </row>
@@ -10395,7 +10398,7 @@
       <c r="H291" s="5">
         <v>84</v>
       </c>
-      <c r="I291" s="15" t="s">
+      <c r="I291" s="16" t="s">
         <v>382</v>
       </c>
     </row>
@@ -10424,7 +10427,7 @@
       <c r="H292" s="5">
         <v>84</v>
       </c>
-      <c r="I292" s="15" t="s">
+      <c r="I292" s="16" t="s">
         <v>383</v>
       </c>
     </row>
@@ -10453,7 +10456,7 @@
       <c r="H293" s="5">
         <v>85</v>
       </c>
-      <c r="I293" s="15" t="s">
+      <c r="I293" s="16" t="s">
         <v>385</v>
       </c>
     </row>
@@ -10482,7 +10485,7 @@
       <c r="H294" s="5">
         <v>85</v>
       </c>
-      <c r="I294" s="15" t="s">
+      <c r="I294" s="16" t="s">
         <v>386</v>
       </c>
     </row>
@@ -10511,7 +10514,7 @@
       <c r="H295" s="5">
         <v>86</v>
       </c>
-      <c r="I295" s="15" t="s">
+      <c r="I295" s="16" t="s">
         <v>388</v>
       </c>
     </row>
@@ -10540,7 +10543,7 @@
       <c r="H296" s="5">
         <v>86</v>
       </c>
-      <c r="I296" s="15" t="s">
+      <c r="I296" s="16" t="s">
         <v>389</v>
       </c>
     </row>
@@ -10569,7 +10572,7 @@
       <c r="H297" s="5">
         <v>87</v>
       </c>
-      <c r="I297" s="15" t="s">
+      <c r="I297" s="16" t="s">
         <v>391</v>
       </c>
     </row>
@@ -10598,7 +10601,7 @@
       <c r="H298" s="5">
         <v>87</v>
       </c>
-      <c r="I298" s="15" t="s">
+      <c r="I298" s="16" t="s">
         <v>392</v>
       </c>
     </row>
@@ -10627,7 +10630,7 @@
       <c r="H299" s="5">
         <v>88</v>
       </c>
-      <c r="I299" s="15" t="s">
+      <c r="I299" s="16" t="s">
         <v>394</v>
       </c>
     </row>
@@ -10656,7 +10659,7 @@
       <c r="H300" s="5">
         <v>88</v>
       </c>
-      <c r="I300" s="15" t="s">
+      <c r="I300" s="16" t="s">
         <v>395</v>
       </c>
     </row>
@@ -10685,7 +10688,7 @@
       <c r="H301" s="5">
         <v>88</v>
       </c>
-      <c r="I301" s="15" t="s">
+      <c r="I301" s="16" t="s">
         <v>396</v>
       </c>
     </row>
@@ -10714,7 +10717,7 @@
       <c r="H302" s="5">
         <v>89</v>
       </c>
-      <c r="I302" s="15" t="s">
+      <c r="I302" s="16" t="s">
         <v>398</v>
       </c>
     </row>
@@ -10743,7 +10746,7 @@
       <c r="H303" s="5">
         <v>89</v>
       </c>
-      <c r="I303" s="15" t="s">
+      <c r="I303" s="16" t="s">
         <v>399</v>
       </c>
     </row>
@@ -10772,7 +10775,7 @@
       <c r="H304" s="5">
         <v>89</v>
       </c>
-      <c r="I304" s="15" t="s">
+      <c r="I304" s="16" t="s">
         <v>400</v>
       </c>
     </row>
@@ -10801,7 +10804,7 @@
       <c r="H305" s="5">
         <v>89</v>
       </c>
-      <c r="I305" s="15" t="s">
+      <c r="I305" s="16" t="s">
         <v>401</v>
       </c>
     </row>
@@ -10830,7 +10833,7 @@
       <c r="H306" s="5">
         <v>90</v>
       </c>
-      <c r="I306" s="15" t="s">
+      <c r="I306" s="16" t="s">
         <v>403</v>
       </c>
     </row>
@@ -10859,7 +10862,7 @@
       <c r="H307" s="5">
         <v>90</v>
       </c>
-      <c r="I307" s="15" t="s">
+      <c r="I307" s="16" t="s">
         <v>404</v>
       </c>
     </row>
@@ -10888,7 +10891,7 @@
       <c r="H308" s="5">
         <v>90</v>
       </c>
-      <c r="I308" s="15" t="s">
+      <c r="I308" s="16" t="s">
         <v>405</v>
       </c>
     </row>
@@ -10917,7 +10920,7 @@
       <c r="H309" s="5">
         <v>91</v>
       </c>
-      <c r="I309" s="15" t="s">
+      <c r="I309" s="16" t="s">
         <v>407</v>
       </c>
     </row>
@@ -10946,7 +10949,7 @@
       <c r="H310" s="5">
         <v>91</v>
       </c>
-      <c r="I310" s="15" t="s">
+      <c r="I310" s="16" t="s">
         <v>408</v>
       </c>
     </row>
@@ -10975,7 +10978,7 @@
       <c r="H311" s="5">
         <v>92</v>
       </c>
-      <c r="I311" s="15" t="s">
+      <c r="I311" s="16" t="s">
         <v>410</v>
       </c>
     </row>
@@ -11004,7 +11007,7 @@
       <c r="H312" s="5">
         <v>92</v>
       </c>
-      <c r="I312" s="15" t="s">
+      <c r="I312" s="16" t="s">
         <v>411</v>
       </c>
     </row>
@@ -11033,7 +11036,7 @@
       <c r="H313" s="5">
         <v>93</v>
       </c>
-      <c r="I313" s="15" t="s">
+      <c r="I313" s="16" t="s">
         <v>413</v>
       </c>
     </row>
@@ -11062,7 +11065,7 @@
       <c r="H314" s="5">
         <v>93</v>
       </c>
-      <c r="I314" s="15" t="s">
+      <c r="I314" s="16" t="s">
         <v>414</v>
       </c>
     </row>
@@ -11091,7 +11094,7 @@
       <c r="H315" s="5">
         <v>93</v>
       </c>
-      <c r="I315" s="15" t="s">
+      <c r="I315" s="16" t="s">
         <v>415</v>
       </c>
     </row>
@@ -11120,7 +11123,7 @@
       <c r="H316" s="5">
         <v>94</v>
       </c>
-      <c r="I316" s="15" t="s">
+      <c r="I316" s="16" t="s">
         <v>417</v>
       </c>
     </row>
@@ -11149,7 +11152,7 @@
       <c r="H317" s="5">
         <v>94</v>
       </c>
-      <c r="I317" s="15" t="s">
+      <c r="I317" s="16" t="s">
         <v>418</v>
       </c>
     </row>
@@ -11178,7 +11181,7 @@
       <c r="H318" s="5">
         <v>94</v>
       </c>
-      <c r="I318" s="15" t="s">
+      <c r="I318" s="16" t="s">
         <v>419</v>
       </c>
     </row>
@@ -11207,7 +11210,7 @@
       <c r="H319" s="5">
         <v>95</v>
       </c>
-      <c r="I319" s="15" t="s">
+      <c r="I319" s="16" t="s">
         <v>421</v>
       </c>
     </row>
@@ -11236,7 +11239,7 @@
       <c r="H320" s="5">
         <v>95</v>
       </c>
-      <c r="I320" s="15" t="s">
+      <c r="I320" s="16" t="s">
         <v>422</v>
       </c>
     </row>
@@ -11265,7 +11268,7 @@
       <c r="H321" s="5">
         <v>96</v>
       </c>
-      <c r="I321" s="15" t="s">
+      <c r="I321" s="16" t="s">
         <v>424</v>
       </c>
     </row>
@@ -11294,7 +11297,7 @@
       <c r="H322" s="5">
         <v>96</v>
       </c>
-      <c r="I322" s="15" t="s">
+      <c r="I322" s="16" t="s">
         <v>425</v>
       </c>
     </row>
@@ -11323,7 +11326,7 @@
       <c r="H323" s="5">
         <v>97</v>
       </c>
-      <c r="I323" s="15" t="s">
+      <c r="I323" s="16" t="s">
         <v>427</v>
       </c>
     </row>
@@ -11352,7 +11355,7 @@
       <c r="H324" s="5">
         <v>97</v>
       </c>
-      <c r="I324" s="15" t="s">
+      <c r="I324" s="16" t="s">
         <v>428</v>
       </c>
     </row>
@@ -11381,7 +11384,7 @@
       <c r="H325" s="5">
         <v>98</v>
       </c>
-      <c r="I325" s="15" t="s">
+      <c r="I325" s="16" t="s">
         <v>430</v>
       </c>
     </row>
@@ -11410,7 +11413,7 @@
       <c r="H326" s="5">
         <v>98</v>
       </c>
-      <c r="I326" s="15" t="s">
+      <c r="I326" s="16" t="s">
         <v>431</v>
       </c>
     </row>
@@ -11439,7 +11442,7 @@
       <c r="H327" s="5">
         <v>98</v>
       </c>
-      <c r="I327" s="15" t="s">
+      <c r="I327" s="16" t="s">
         <v>432</v>
       </c>
     </row>
@@ -11468,7 +11471,7 @@
       <c r="H328" s="5">
         <v>99</v>
       </c>
-      <c r="I328" s="15" t="s">
+      <c r="I328" s="16" t="s">
         <v>434</v>
       </c>
     </row>
@@ -11497,7 +11500,7 @@
       <c r="H329" s="5">
         <v>99</v>
       </c>
-      <c r="I329" s="15" t="s">
+      <c r="I329" s="16" t="s">
         <v>435</v>
       </c>
     </row>
@@ -11526,7 +11529,7 @@
       <c r="H330" s="5">
         <v>99</v>
       </c>
-      <c r="I330" s="15" t="s">
+      <c r="I330" s="16" t="s">
         <v>436</v>
       </c>
     </row>
@@ -11555,7 +11558,7 @@
       <c r="H331" s="5">
         <v>100</v>
       </c>
-      <c r="I331" s="15" t="s">
+      <c r="I331" s="16" t="s">
         <v>438</v>
       </c>
     </row>
@@ -11584,7 +11587,7 @@
       <c r="H332" s="5">
         <v>100</v>
       </c>
-      <c r="I332" s="15" t="s">
+      <c r="I332" s="16" t="s">
         <v>439</v>
       </c>
     </row>
@@ -11613,7 +11616,7 @@
       <c r="H333" s="5">
         <v>101</v>
       </c>
-      <c r="I333" s="15" t="s">
+      <c r="I333" s="16" t="s">
         <v>441</v>
       </c>
     </row>
@@ -11642,7 +11645,7 @@
       <c r="H334" s="5">
         <v>101</v>
       </c>
-      <c r="I334" s="15" t="s">
+      <c r="I334" s="16" t="s">
         <v>442</v>
       </c>
     </row>
@@ -11671,7 +11674,7 @@
       <c r="H335" s="5">
         <v>102</v>
       </c>
-      <c r="I335" s="15" t="s">
+      <c r="I335" s="16" t="s">
         <v>444</v>
       </c>
     </row>
@@ -11700,7 +11703,7 @@
       <c r="H336" s="5">
         <v>102</v>
       </c>
-      <c r="I336" s="15" t="s">
+      <c r="I336" s="16" t="s">
         <v>445</v>
       </c>
     </row>
@@ -11729,7 +11732,7 @@
       <c r="H337" s="5">
         <v>103</v>
       </c>
-      <c r="I337" s="15" t="s">
+      <c r="I337" s="16" t="s">
         <v>447</v>
       </c>
     </row>
@@ -11758,7 +11761,7 @@
       <c r="H338" s="5">
         <v>103</v>
       </c>
-      <c r="I338" s="15" t="s">
+      <c r="I338" s="16" t="s">
         <v>448</v>
       </c>
     </row>
@@ -11787,7 +11790,7 @@
       <c r="H339" s="5">
         <v>104</v>
       </c>
-      <c r="I339" s="15" t="s">
+      <c r="I339" s="16" t="s">
         <v>450</v>
       </c>
     </row>
@@ -11816,7 +11819,7 @@
       <c r="H340" s="5">
         <v>104</v>
       </c>
-      <c r="I340" s="15" t="s">
+      <c r="I340" s="16" t="s">
         <v>451</v>
       </c>
     </row>
@@ -11845,7 +11848,7 @@
       <c r="H341" s="5">
         <v>105</v>
       </c>
-      <c r="I341" s="15" t="s">
+      <c r="I341" s="16" t="s">
         <v>453</v>
       </c>
     </row>
@@ -11874,7 +11877,7 @@
       <c r="H342" s="5">
         <v>105</v>
       </c>
-      <c r="I342" s="15" t="s">
+      <c r="I342" s="16" t="s">
         <v>454</v>
       </c>
     </row>
@@ -11903,7 +11906,7 @@
       <c r="H343" s="5">
         <v>106</v>
       </c>
-      <c r="I343" s="15" t="s">
+      <c r="I343" s="16" t="s">
         <v>456</v>
       </c>
     </row>
@@ -11932,7 +11935,7 @@
       <c r="H344" s="5">
         <v>106</v>
       </c>
-      <c r="I344" s="15" t="s">
+      <c r="I344" s="16" t="s">
         <v>457</v>
       </c>
     </row>
@@ -11961,7 +11964,7 @@
       <c r="H345" s="5">
         <v>107</v>
       </c>
-      <c r="I345" s="15" t="s">
+      <c r="I345" s="16" t="s">
         <v>459</v>
       </c>
     </row>
@@ -11990,7 +11993,7 @@
       <c r="H346" s="5">
         <v>107</v>
       </c>
-      <c r="I346" s="15" t="s">
+      <c r="I346" s="16" t="s">
         <v>460</v>
       </c>
     </row>
@@ -12019,7 +12022,7 @@
       <c r="H347" s="5">
         <v>107</v>
       </c>
-      <c r="I347" s="15" t="s">
+      <c r="I347" s="16" t="s">
         <v>461</v>
       </c>
     </row>
@@ -12048,7 +12051,7 @@
       <c r="H348" s="5">
         <v>108</v>
       </c>
-      <c r="I348" s="15" t="s">
+      <c r="I348" s="16" t="s">
         <v>463</v>
       </c>
     </row>
@@ -12075,7 +12078,7 @@
       <c r="H349" s="5">
         <v>108</v>
       </c>
-      <c r="I349" s="15" t="s">
+      <c r="I349" s="16" t="s">
         <v>464</v>
       </c>
     </row>
@@ -12104,7 +12107,7 @@
       <c r="H350" s="5">
         <v>109</v>
       </c>
-      <c r="I350" s="15" t="s">
+      <c r="I350" s="16" t="s">
         <v>466</v>
       </c>
     </row>
@@ -12131,7 +12134,7 @@
       <c r="H351" s="5">
         <v>109</v>
       </c>
-      <c r="I351" s="15" t="s">
+      <c r="I351" s="16" t="s">
         <v>467</v>
       </c>
     </row>
@@ -12158,7 +12161,7 @@
       <c r="H352" s="5">
         <v>109</v>
       </c>
-      <c r="I352" s="15" t="s">
+      <c r="I352" s="16" t="s">
         <v>468</v>
       </c>
     </row>
@@ -12185,7 +12188,7 @@
       <c r="H353" s="5">
         <v>109</v>
       </c>
-      <c r="I353" s="15" t="s">
+      <c r="I353" s="16" t="s">
         <v>469</v>
       </c>
     </row>
@@ -12214,7 +12217,7 @@
       <c r="H354" s="5">
         <v>110</v>
       </c>
-      <c r="I354" s="15" t="s">
+      <c r="I354" s="16" t="s">
         <v>471</v>
       </c>
     </row>
@@ -12241,7 +12244,7 @@
       <c r="H355" s="5">
         <v>110</v>
       </c>
-      <c r="I355" s="15" t="s">
+      <c r="I355" s="16" t="s">
         <v>472</v>
       </c>
     </row>
@@ -12270,7 +12273,7 @@
       <c r="H356" s="5">
         <v>111</v>
       </c>
-      <c r="I356" s="15" t="s">
+      <c r="I356" s="16" t="s">
         <v>474</v>
       </c>
     </row>
@@ -12297,7 +12300,7 @@
       <c r="H357" s="5">
         <v>111</v>
       </c>
-      <c r="I357" s="15" t="s">
+      <c r="I357" s="16" t="s">
         <v>475</v>
       </c>
     </row>
@@ -12326,7 +12329,7 @@
       <c r="H358" s="5">
         <v>112</v>
       </c>
-      <c r="I358" s="15" t="s">
+      <c r="I358" s="16" t="s">
         <v>477</v>
       </c>
     </row>
@@ -12353,7 +12356,7 @@
       <c r="H359" s="5">
         <v>112</v>
       </c>
-      <c r="I359" s="15" t="s">
+      <c r="I359" s="16" t="s">
         <v>478</v>
       </c>
     </row>
@@ -12380,7 +12383,7 @@
       <c r="H360" s="5">
         <v>112</v>
       </c>
-      <c r="I360" s="15" t="s">
+      <c r="I360" s="16" t="s">
         <v>479</v>
       </c>
     </row>
@@ -12407,7 +12410,7 @@
       <c r="H361" s="5">
         <v>112</v>
       </c>
-      <c r="I361" s="15" t="s">
+      <c r="I361" s="16" t="s">
         <v>480</v>
       </c>
     </row>
@@ -12436,7 +12439,7 @@
       <c r="H362" s="5">
         <v>113</v>
       </c>
-      <c r="I362" s="15" t="s">
+      <c r="I362" s="16" t="s">
         <v>482</v>
       </c>
     </row>
@@ -12463,7 +12466,7 @@
       <c r="H363" s="5">
         <v>113</v>
       </c>
-      <c r="I363" s="15" t="s">
+      <c r="I363" s="16" t="s">
         <v>483</v>
       </c>
     </row>
@@ -12492,7 +12495,7 @@
       <c r="H364" s="11">
         <v>114</v>
       </c>
-      <c r="I364" s="17" t="s">
+      <c r="I364" s="18" t="s">
         <v>485</v>
       </c>
     </row>
@@ -12519,7 +12522,7 @@
       <c r="H365" s="11">
         <v>114</v>
       </c>
-      <c r="I365" s="17" t="s">
+      <c r="I365" s="18" t="s">
         <v>486</v>
       </c>
     </row>

</xml_diff>